<commit_message>
feat(iso27001): improved model with overlay, expanded mappings
</commit_message>
<xml_diff>
--- a/project/excel/iso27001.xlsx
+++ b/project/excel/iso27001.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL1"/>
+  <dimension ref="A1:AT1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,185 +456,225 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>top_management</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>governing_body</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>leadership_commitment_evidence</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>scope_statement</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>scope_boundaries</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>scope_exclusions</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>interfaces_and_dependencies</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>processes_and_interactions</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>context_internal_issues</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>context_external_issues</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>interested_parties</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>information_security_policy</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>objectives</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>risks_and_opportunities_actions</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>planned_changes</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>externally_provided_services</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
         <is>
           <t>risk_assessment_process</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>risk_treatment_process</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>statement_of_applicability</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>controls</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>roles</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>resources</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>competence_records</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>awareness_program</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>communication_plan</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>documented_information_register</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>operational_procedures</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>risk_assessments</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>risk_treatment_plans</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>monitoring_program</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>internal_audits</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>management_reviews</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>nonconformities</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>corrective_actions</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>improvements</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>certification_status</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>certification_body</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>certification_date</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>recertification_date</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -757,7 +797,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="6">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"confidentiality,integrity,availability"</formula1>
+    </dataValidation>
     <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"rare,unlikely,possible,likely,almost_certain"</formula1>
     </dataValidation>
@@ -784,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -800,95 +843,125 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>annex_a_omission_verification</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>soa_template</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>approval_workflow</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>document_type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>author</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>approved_by</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>approved_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>effective_date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>review_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>classification</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>retention_period</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -896,7 +969,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"policy,procedure,standard,guideline,record,plan,report"</formula1>
     </dataValidation>
   </dataValidations>
@@ -910,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1026,30 +1099,55 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -1074,7 +1172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1165,30 +1263,55 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -1471,7 +1594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1577,30 +1700,55 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -1622,7 +1770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1713,30 +1861,55 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -1758,7 +1931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1824,30 +1997,55 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -2021,7 +2219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2112,30 +2310,55 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -2157,7 +2380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2223,30 +2446,55 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -2339,7 +2587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG1"/>
+  <dimension ref="A1:AL1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2480,37 +2728,65 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"internal,external_second_party,external_third_party,surveillance,recertification,combined"</formula1>
+    </dataValidation>
     <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"policy,procedure,standard,guideline,record,plan,report"</formula1>
     </dataValidation>
@@ -2525,7 +2801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2616,30 +2892,55 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -2772,7 +3073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AJ1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2803,115 +3104,155 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>interested_party_feedback</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>performance_trends</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>audit_results_summary</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>risk_assessment_results</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>risk_treatment_status</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>risks_and_opportunities_changes</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>improvement_opportunities</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>decisions</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>action_items</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>next_review_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_type</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>author</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>approved_by</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>approved_date</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>effective_date</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>classification</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>retention_period</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -2919,7 +3260,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"policy,procedure,standard,guideline,record,plan,report"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3150,7 +3491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3171,40 +3512,50 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>addressed_requirements</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>climate_change_related_requirements</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>communication_needs</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>contact_information</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -3620,6 +3971,14 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"very_low,low,medium,high,critical"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"confidentiality,integrity,availability"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3630,7 +3989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3666,98 +4025,141 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>last_policy_review_date</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>next_policy_review_date</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>related_topic_policies</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>integrated_management_systems</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_type</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>author</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>approved_by</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>approved_date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>effective_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>review_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>classification</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>retention_period</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"iso_iec_27001,iso_iec_27701,iso_iec_27017,iso_iec_27018,iso_iec_42001,iso_9001,iso_14001,iso_22301,iso_iec_20000_1,iso_31000"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"policy,procedure,standard,guideline,record,plan,report"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3771,7 +4173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3852,30 +4254,55 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -3978,7 +4405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4044,30 +4471,35 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>objective_resources_required</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -4084,7 +4516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:AD1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4185,30 +4617,55 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -4230,7 +4687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:AD1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4331,30 +4788,55 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
+          <t>distribution_controls</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>storage_and_preservation</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>change_control_method</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>external_origin</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>external_origin_source</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>version</t>
         </is>

</xml_diff>